<commit_message>
Atualização automática leitura Parcial_Americana.xlsx
</commit_message>
<xml_diff>
--- a/dashboard/leitura/Parcial_Americana.xlsx
+++ b/dashboard/leitura/Parcial_Americana.xlsx
@@ -634,13 +634,13 @@
         <v>789</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>653</v>
+        <v>684</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>136</v>
+        <v>105</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>82.76000000000001</v>
+        <v>86.69</v>
       </c>
     </row>
     <row r="9">
@@ -665,58 +665,58 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>EDUARDO DE ABREU BARBOSA</t>
+          <t>EUGENIO RESERVA</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>999</v>
+        <v>655</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>910</v>
+        <v>597</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>89</v>
+        <v>58</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>91.09</v>
+        <v>91.15000000000001</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>EUGENIO RESERVA</t>
+          <t>WILTON DO CARMO MORIS ARAUJO</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>655</v>
+        <v>472</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>597</v>
+        <v>432</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>91.15000000000001</v>
+        <v>91.53</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>WILTON DO CARMO MORIS ARAUJO</t>
+          <t>EDUARDO DE ABREU BARBOSA</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>472</v>
+        <v>999</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>432</v>
+        <v>942</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>40</v>
+        <v>57</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>91.53</v>
+        <v>94.29000000000001</v>
       </c>
     </row>
     <row r="13">

</xml_diff>